<commit_message>
Correct Turkish UI copy and prevent missing Turkish glyphs
</commit_message>
<xml_diff>
--- a/docs/reports/bom/ORNEK_BOM_URUN_AGACI.xlsx
+++ b/docs/reports/bom/ORNEK_BOM_URUN_AGACI.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T11:06:26+03:00</t>
+          <t>2026-10-12T11:46:50+03:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -518,7 +518,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BOM dışı hariç</t>
+          <t>BOM dışında bırakılanlar hariç</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -667,7 +667,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T11:06:26+03:00</t>
+          <t>2026-10-12T11:46:50+03:00</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -690,7 +690,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>BOM dışı hariç</t>
+          <t>BOM dışında bırakılanlar hariç</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>

</xml_diff>